<commit_message>
Clean up activities and confirm back navigation to Personal Recommendations
</commit_message>
<xml_diff>
--- a/frontend/ml/recommendations.xlsx
+++ b/frontend/ml/recommendations.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ML_Recommendations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,48 +415,39 @@
   </sheetPr>
   <dimension ref="A1:G1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>emotion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>recommended_activities</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>recommended_games</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>recommended_music</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>recommended_videos</t>
         </is>
@@ -854,7 +841,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1261,7 +1248,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1779,7 +1766,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2408,7 +2395,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2741,7 +2728,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3481,7 +3468,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3703,7 +3690,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4036,7 +4023,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4184,7 +4171,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -4221,7 +4208,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4517,7 +4504,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4554,7 +4541,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5109,7 +5096,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5220,7 +5207,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5331,7 +5318,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5775,7 +5762,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -5923,7 +5910,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6071,7 +6058,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6515,7 +6502,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -6700,7 +6687,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -6959,7 +6946,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -7255,7 +7242,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -7292,7 +7279,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -7329,7 +7316,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -7440,7 +7427,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -7699,7 +7686,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -8624,7 +8611,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -9031,7 +9018,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -9179,7 +9166,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -9586,7 +9573,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -10030,7 +10017,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -10511,7 +10498,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -11103,7 +11090,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11251,7 +11238,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11917,7 +11904,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -11991,7 +11978,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12065,7 +12052,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12324,7 +12311,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -13693,7 +13680,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -14433,7 +14420,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -14507,7 +14494,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -14544,7 +14531,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E382" t="inlineStr">
@@ -14581,7 +14568,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
@@ -14729,7 +14716,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -15210,7 +15197,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
@@ -15321,7 +15308,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
@@ -15543,7 +15530,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -15802,7 +15789,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
@@ -16098,7 +16085,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
@@ -16172,7 +16159,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
@@ -16246,7 +16233,7 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
@@ -16431,7 +16418,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
@@ -16468,7 +16455,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -16875,7 +16862,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
@@ -17171,7 +17158,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
@@ -17652,7 +17639,7 @@
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
@@ -18355,7 +18342,7 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E485" t="inlineStr">
@@ -18429,7 +18416,7 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E487" t="inlineStr">
@@ -19354,7 +19341,7 @@
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E512" t="inlineStr">
@@ -19391,7 +19378,7 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
@@ -19724,7 +19711,7 @@
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E522" t="inlineStr">
@@ -20205,7 +20192,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
@@ -21352,7 +21339,7 @@
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
@@ -21426,7 +21413,7 @@
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
@@ -21463,7 +21450,7 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
@@ -22240,7 +22227,7 @@
       </c>
       <c r="D590" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E590" t="inlineStr">
@@ -22277,7 +22264,7 @@
       </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E591" t="inlineStr">
@@ -22388,7 +22375,7 @@
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E594" t="inlineStr">
@@ -22573,7 +22560,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
@@ -22758,7 +22745,7 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
@@ -23350,7 +23337,7 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
@@ -23535,7 +23522,7 @@
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
@@ -23646,7 +23633,7 @@
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
@@ -24608,7 +24595,7 @@
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E654" t="inlineStr">
@@ -24793,7 +24780,7 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
@@ -24830,7 +24817,7 @@
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
@@ -25681,7 +25668,7 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E683" t="inlineStr">
@@ -25718,7 +25705,7 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
@@ -25977,7 +25964,7 @@
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E691" t="inlineStr">
@@ -26310,7 +26297,7 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
@@ -26791,7 +26778,7 @@
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
@@ -27494,7 +27481,7 @@
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
@@ -27642,7 +27629,7 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
@@ -27716,7 +27703,7 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
@@ -28049,7 +28036,7 @@
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
@@ -28271,7 +28258,7 @@
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E753" t="inlineStr">
@@ -28567,7 +28554,7 @@
       </c>
       <c r="D761" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E761" t="inlineStr">
@@ -28604,7 +28591,7 @@
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E762" t="inlineStr">
@@ -28715,7 +28702,7 @@
       </c>
       <c r="D765" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E765" t="inlineStr">
@@ -28789,7 +28776,7 @@
       </c>
       <c r="D767" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E767" t="inlineStr">
@@ -28937,7 +28924,7 @@
       </c>
       <c r="D771" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E771" t="inlineStr">
@@ -29048,7 +29035,7 @@
       </c>
       <c r="D774" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E774" t="inlineStr">
@@ -29233,7 +29220,7 @@
       </c>
       <c r="D779" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E779" t="inlineStr">
@@ -29603,7 +29590,7 @@
       </c>
       <c r="D789" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E789" t="inlineStr">
@@ -30010,7 +29997,7 @@
       </c>
       <c r="D800" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E800" t="inlineStr">
@@ -30639,7 +30626,7 @@
       </c>
       <c r="D817" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E817" t="inlineStr">
@@ -30972,7 +30959,7 @@
       </c>
       <c r="D826" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E826" t="inlineStr">
@@ -31305,7 +31292,7 @@
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E835" t="inlineStr">
@@ -31490,7 +31477,7 @@
       </c>
       <c r="D840" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E840" t="inlineStr">
@@ -31527,7 +31514,7 @@
       </c>
       <c r="D841" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E841" t="inlineStr">
@@ -31601,7 +31588,7 @@
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E843" t="inlineStr">
@@ -31860,7 +31847,7 @@
       </c>
       <c r="D850" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E850" t="inlineStr">
@@ -31971,7 +31958,7 @@
       </c>
       <c r="D853" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E853" t="inlineStr">
@@ -32008,7 +31995,7 @@
       </c>
       <c r="D854" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E854" t="inlineStr">
@@ -32193,7 +32180,7 @@
       </c>
       <c r="D859" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E859" t="inlineStr">
@@ -32267,7 +32254,7 @@
       </c>
       <c r="D861" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E861" t="inlineStr">
@@ -32526,7 +32513,7 @@
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
@@ -32711,7 +32698,7 @@
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
@@ -32748,7 +32735,7 @@
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E874" t="inlineStr">
@@ -33229,7 +33216,7 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
@@ -33599,7 +33586,7 @@
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E897" t="inlineStr">
@@ -33932,7 +33919,7 @@
       </c>
       <c r="D906" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E906" t="inlineStr">
@@ -33969,7 +33956,7 @@
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E907" t="inlineStr">
@@ -34154,7 +34141,7 @@
       </c>
       <c r="D912" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E912" t="inlineStr">
@@ -34265,7 +34252,7 @@
       </c>
       <c r="D915" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E915" t="inlineStr">
@@ -34339,7 +34326,7 @@
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E917" t="inlineStr">
@@ -34376,7 +34363,7 @@
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E918" t="inlineStr">
@@ -35227,7 +35214,7 @@
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E941" t="inlineStr">
@@ -35449,7 +35436,7 @@
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
@@ -35486,7 +35473,7 @@
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
@@ -36522,7 +36509,7 @@
       </c>
       <c r="D976" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E976" t="inlineStr">
@@ -36596,7 +36583,7 @@
       </c>
       <c r="D978" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E978" t="inlineStr">
@@ -36633,7 +36620,7 @@
       </c>
       <c r="D979" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E979" t="inlineStr">
@@ -36892,7 +36879,7 @@
       </c>
       <c r="D986" t="inlineStr">
         <is>
-          <t>baby_bonding, journaling, affirmation_activity</t>
+          <t>baby_mood, journaling, affirmation_activity</t>
         </is>
       </c>
       <c r="E986" t="inlineStr">
@@ -37373,7 +37360,7 @@
       </c>
       <c r="D999" t="inlineStr">
         <is>
-          <t>baby_bonding, breathing_478, colouring</t>
+          <t>baby_mood, breathing_478, colouring</t>
         </is>
       </c>
       <c r="E999" t="inlineStr">

</xml_diff>